<commit_message>
Laminas de salud y educacion con las cifras corregidas
Salud: tasas por sexo recalculadas (el denominador estaba al doble, ver PIDR
1e3d5cfa) y bandas de edad con los denominadores demograficos nuevos.
Incluye las laminas regionales por sexo y tramo de edad que el sitio pasa a
mostrar, y las nacionales de valor, serie e interregional.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nb4kJtgDC9tzWdETyfNewy
</commit_message>
<xml_diff>
--- a/output/graficos_regionales_sexo_edad/plot_historia_nacional_s_fonasa_a_2021_nacional.xlsx
+++ b/output/graficos_regionales_sexo_edad/plot_historia_nacional_s_fonasa_a_2021_nacional.xlsx
@@ -40,7 +40,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-08-28 15:08</t>
+    <t xml:space="preserve">2026-08-29 05:46</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -480,7 +480,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>43.03</v>
+        <v>86.07</v>
       </c>
     </row>
     <row r="3">
@@ -491,7 +491,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>41.66</v>
+        <v>83.32</v>
       </c>
     </row>
     <row r="4">
@@ -502,7 +502,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>42.79</v>
+        <v>85.58</v>
       </c>
     </row>
     <row r="5">
@@ -513,7 +513,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>42.93</v>
+        <v>85.86</v>
       </c>
     </row>
     <row r="6">
@@ -524,7 +524,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>40.32</v>
+        <v>80.65</v>
       </c>
     </row>
     <row r="7">
@@ -535,7 +535,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>39.01</v>
+        <v>78.02</v>
       </c>
     </row>
     <row r="8">
@@ -546,7 +546,7 @@
         <v>4</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>40.34</v>
+        <v>80.68</v>
       </c>
     </row>
     <row r="9">
@@ -557,7 +557,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>40.56</v>
+        <v>81.12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>